<commit_message>
Till Top K Frequent Elements
</commit_message>
<xml_diff>
--- a/Java_Developer_Roadmap.xlsx
+++ b/Java_Developer_Roadmap.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDAE2EC6-B12E-45D9-B1A7-4701C497F8BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB2B5F8-6D0F-48F9-9B42-AAE6FC9CFB8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="288">
   <si>
     <t>Level</t>
   </si>
@@ -1797,7 +1797,9 @@
       <c r="D32" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E32" s="3"/>
+      <c r="E32" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">

</xml_diff>

<commit_message>
Till Longest Consecutive Sequence
</commit_message>
<xml_diff>
--- a/Java_Developer_Roadmap.xlsx
+++ b/Java_Developer_Roadmap.xlsx
@@ -1,15 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB2B5F8-6D0F-48F9-9B42-AAE6FC9CFB8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
-    <sheet name="Roadmap" sheetId="1" r:id="rId1"/>
-    <sheet name="Topics &amp; Subtopics" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Roadmap" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Topics &amp; Subtopics" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">'Topics &amp; Subtopics'!$A$1:$C$29</definedName>
@@ -19,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="288">
   <si>
     <t>Level</t>
   </si>
@@ -888,19 +887,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1246,9 +1245,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E220"/>
-  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -1563,7 +1562,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
@@ -1580,7 +1579,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
@@ -1597,7 +1596,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>26</v>
       </c>
@@ -1614,7 +1613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
@@ -1631,7 +1630,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
@@ -1648,7 +1647,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>26</v>
       </c>
@@ -1665,7 +1664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
@@ -1682,7 +1681,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
@@ -1699,7 +1698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -1716,7 +1715,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -1733,7 +1732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>26</v>
       </c>
@@ -1750,7 +1749,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>26</v>
       </c>
@@ -1767,7 +1766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -1784,7 +1783,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -1801,7 +1800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>26</v>
       </c>
@@ -1814,9 +1813,11 @@
       <c r="D33" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E33" s="3"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E33" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>26</v>
       </c>
@@ -1831,7 +1832,7 @@
       </c>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>26</v>
       </c>
@@ -1846,7 +1847,7 @@
       </c>
       <c r="E35" s="3"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>26</v>
       </c>
@@ -1861,7 +1862,7 @@
       </c>
       <c r="E36" s="3"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>26</v>
       </c>
@@ -1876,7 +1877,7 @@
       </c>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>26</v>
       </c>
@@ -1891,7 +1892,7 @@
       </c>
       <c r="E38" s="3"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>26</v>
       </c>
@@ -1906,7 +1907,7 @@
       </c>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>26</v>
       </c>
@@ -1921,7 +1922,7 @@
       </c>
       <c r="E40" s="3"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>26</v>
       </c>
@@ -1936,7 +1937,7 @@
       </c>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>26</v>
       </c>
@@ -1951,7 +1952,7 @@
       </c>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>26</v>
       </c>
@@ -1966,7 +1967,7 @@
       </c>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>26</v>
       </c>
@@ -1981,7 +1982,7 @@
       </c>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>26</v>
       </c>
@@ -1996,7 +1997,7 @@
       </c>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2011,7 +2012,7 @@
       </c>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>26</v>
       </c>
@@ -2026,7 +2027,7 @@
       </c>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>26</v>
       </c>
@@ -2041,7 +2042,7 @@
       </c>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>61</v>
       </c>
@@ -2056,7 +2057,7 @@
       </c>
       <c r="E49" s="3"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>61</v>
       </c>
@@ -2071,7 +2072,7 @@
       </c>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>61</v>
       </c>
@@ -2086,7 +2087,7 @@
       </c>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>61</v>
       </c>
@@ -2101,7 +2102,7 @@
       </c>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>61</v>
       </c>
@@ -2116,7 +2117,7 @@
       </c>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>61</v>
       </c>
@@ -2131,7 +2132,7 @@
       </c>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>61</v>
       </c>
@@ -2146,7 +2147,7 @@
       </c>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>61</v>
       </c>
@@ -2161,7 +2162,7 @@
       </c>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>61</v>
       </c>
@@ -2176,7 +2177,7 @@
       </c>
       <c r="E57" s="3"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>61</v>
       </c>
@@ -2191,7 +2192,7 @@
       </c>
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>61</v>
       </c>
@@ -2206,7 +2207,7 @@
       </c>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>61</v>
       </c>
@@ -2221,7 +2222,7 @@
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>61</v>
       </c>
@@ -2236,7 +2237,7 @@
       </c>
       <c r="E61" s="3"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -2251,7 +2252,7 @@
       </c>
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -2266,7 +2267,7 @@
       </c>
       <c r="E63" s="3"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>61</v>
       </c>
@@ -2281,7 +2282,7 @@
       </c>
       <c r="E64" s="3"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>61</v>
       </c>
@@ -2296,7 +2297,7 @@
       </c>
       <c r="E65" s="3"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>61</v>
       </c>
@@ -2311,7 +2312,7 @@
       </c>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>61</v>
       </c>
@@ -2326,7 +2327,7 @@
       </c>
       <c r="E67" s="3"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>61</v>
       </c>
@@ -2341,7 +2342,7 @@
       </c>
       <c r="E68" s="3"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>61</v>
       </c>
@@ -2356,7 +2357,7 @@
       </c>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>61</v>
       </c>
@@ -2371,7 +2372,7 @@
       </c>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>61</v>
       </c>
@@ -2386,7 +2387,7 @@
       </c>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>61</v>
       </c>
@@ -2401,7 +2402,7 @@
       </c>
       <c r="E72" s="3"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>61</v>
       </c>
@@ -2416,7 +2417,7 @@
       </c>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>61</v>
       </c>
@@ -2431,7 +2432,7 @@
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>61</v>
       </c>
@@ -2446,7 +2447,7 @@
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>61</v>
       </c>
@@ -2461,7 +2462,7 @@
       </c>
       <c r="E76" s="3"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>61</v>
       </c>
@@ -2476,7 +2477,7 @@
       </c>
       <c r="E77" s="3"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>61</v>
       </c>
@@ -2491,7 +2492,7 @@
       </c>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>61</v>
       </c>
@@ -2506,7 +2507,7 @@
       </c>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>61</v>
       </c>
@@ -2521,7 +2522,7 @@
       </c>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>61</v>
       </c>
@@ -2536,7 +2537,7 @@
       </c>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>61</v>
       </c>
@@ -2551,7 +2552,7 @@
       </c>
       <c r="E82" s="3"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>61</v>
       </c>
@@ -2566,7 +2567,7 @@
       </c>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>61</v>
       </c>
@@ -2581,7 +2582,7 @@
       </c>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>61</v>
       </c>
@@ -2596,7 +2597,7 @@
       </c>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>61</v>
       </c>
@@ -2611,7 +2612,7 @@
       </c>
       <c r="E86" s="3"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>61</v>
       </c>
@@ -2626,7 +2627,7 @@
       </c>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>61</v>
       </c>
@@ -2641,7 +2642,7 @@
       </c>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>61</v>
       </c>
@@ -2656,7 +2657,7 @@
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>61</v>
       </c>
@@ -2671,7 +2672,7 @@
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>61</v>
       </c>
@@ -2686,7 +2687,7 @@
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>61</v>
       </c>
@@ -2701,7 +2702,7 @@
       </c>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>61</v>
       </c>
@@ -2716,7 +2717,7 @@
       </c>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>61</v>
       </c>
@@ -2731,7 +2732,7 @@
       </c>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>61</v>
       </c>
@@ -2746,7 +2747,7 @@
       </c>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>61</v>
       </c>
@@ -2761,7 +2762,7 @@
       </c>
       <c r="E96" s="3"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>61</v>
       </c>
@@ -2776,7 +2777,7 @@
       </c>
       <c r="E97" s="3"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>61</v>
       </c>
@@ -2791,7 +2792,7 @@
       </c>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>61</v>
       </c>
@@ -2806,7 +2807,7 @@
       </c>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>61</v>
       </c>
@@ -2821,7 +2822,7 @@
       </c>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>120</v>
       </c>
@@ -2836,7 +2837,7 @@
       </c>
       <c r="E101" s="3"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>120</v>
       </c>
@@ -2851,7 +2852,7 @@
       </c>
       <c r="E102" s="3"/>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>120</v>
       </c>
@@ -2866,7 +2867,7 @@
       </c>
       <c r="E103" s="3"/>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>120</v>
       </c>
@@ -2881,7 +2882,7 @@
       </c>
       <c r="E104" s="3"/>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>120</v>
       </c>
@@ -2896,7 +2897,7 @@
       </c>
       <c r="E105" s="3"/>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>120</v>
       </c>
@@ -2911,7 +2912,7 @@
       </c>
       <c r="E106" s="3"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>120</v>
       </c>
@@ -2926,7 +2927,7 @@
       </c>
       <c r="E107" s="3"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>120</v>
       </c>
@@ -2941,7 +2942,7 @@
       </c>
       <c r="E108" s="3"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>120</v>
       </c>
@@ -2956,7 +2957,7 @@
       </c>
       <c r="E109" s="3"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>120</v>
       </c>
@@ -2971,7 +2972,7 @@
       </c>
       <c r="E110" s="3"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>120</v>
       </c>
@@ -2986,7 +2987,7 @@
       </c>
       <c r="E111" s="3"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>120</v>
       </c>
@@ -3001,7 +3002,7 @@
       </c>
       <c r="E112" s="3"/>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>120</v>
       </c>
@@ -3016,7 +3017,7 @@
       </c>
       <c r="E113" s="3"/>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>120</v>
       </c>
@@ -3031,7 +3032,7 @@
       </c>
       <c r="E114" s="3"/>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>120</v>
       </c>
@@ -3046,7 +3047,7 @@
       </c>
       <c r="E115" s="3"/>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>120</v>
       </c>
@@ -3061,7 +3062,7 @@
       </c>
       <c r="E116" s="3"/>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>120</v>
       </c>
@@ -3076,7 +3077,7 @@
       </c>
       <c r="E117" s="3"/>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>120</v>
       </c>
@@ -3091,7 +3092,7 @@
       </c>
       <c r="E118" s="3"/>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>120</v>
       </c>
@@ -3106,7 +3107,7 @@
       </c>
       <c r="E119" s="3"/>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>120</v>
       </c>
@@ -3121,7 +3122,7 @@
       </c>
       <c r="E120" s="3"/>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>120</v>
       </c>
@@ -3136,7 +3137,7 @@
       </c>
       <c r="E121" s="3"/>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>120</v>
       </c>
@@ -3151,7 +3152,7 @@
       </c>
       <c r="E122" s="3"/>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>120</v>
       </c>
@@ -3166,7 +3167,7 @@
       </c>
       <c r="E123" s="3"/>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>120</v>
       </c>
@@ -3181,7 +3182,7 @@
       </c>
       <c r="E124" s="3"/>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>120</v>
       </c>
@@ -3196,7 +3197,7 @@
       </c>
       <c r="E125" s="3"/>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>120</v>
       </c>
@@ -3211,7 +3212,7 @@
       </c>
       <c r="E126" s="3"/>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>120</v>
       </c>
@@ -3226,7 +3227,7 @@
       </c>
       <c r="E127" s="3"/>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>120</v>
       </c>
@@ -3241,7 +3242,7 @@
       </c>
       <c r="E128" s="3"/>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>120</v>
       </c>
@@ -3256,7 +3257,7 @@
       </c>
       <c r="E129" s="3"/>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>120</v>
       </c>
@@ -3271,7 +3272,7 @@
       </c>
       <c r="E130" s="3"/>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>120</v>
       </c>
@@ -3286,7 +3287,7 @@
       </c>
       <c r="E131" s="3"/>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>120</v>
       </c>
@@ -3301,7 +3302,7 @@
       </c>
       <c r="E132" s="3"/>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>158</v>
       </c>
@@ -3316,7 +3317,7 @@
       </c>
       <c r="E133" s="3"/>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>158</v>
       </c>
@@ -3331,7 +3332,7 @@
       </c>
       <c r="E134" s="3"/>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>158</v>
       </c>
@@ -3346,7 +3347,7 @@
       </c>
       <c r="E135" s="3"/>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>158</v>
       </c>
@@ -3361,7 +3362,7 @@
       </c>
       <c r="E136" s="3"/>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>158</v>
       </c>
@@ -3376,7 +3377,7 @@
       </c>
       <c r="E137" s="3"/>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>158</v>
       </c>
@@ -3391,7 +3392,7 @@
       </c>
       <c r="E138" s="3"/>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>158</v>
       </c>
@@ -3406,7 +3407,7 @@
       </c>
       <c r="E139" s="3"/>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>158</v>
       </c>
@@ -3421,7 +3422,7 @@
       </c>
       <c r="E140" s="3"/>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>158</v>
       </c>
@@ -3436,7 +3437,7 @@
       </c>
       <c r="E141" s="3"/>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>158</v>
       </c>
@@ -3451,7 +3452,7 @@
       </c>
       <c r="E142" s="3"/>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>158</v>
       </c>
@@ -3466,7 +3467,7 @@
       </c>
       <c r="E143" s="3"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>158</v>
       </c>
@@ -3481,7 +3482,7 @@
       </c>
       <c r="E144" s="3"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>158</v>
       </c>
@@ -3496,7 +3497,7 @@
       </c>
       <c r="E145" s="3"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>158</v>
       </c>
@@ -3511,7 +3512,7 @@
       </c>
       <c r="E146" s="3"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>158</v>
       </c>
@@ -3526,7 +3527,7 @@
       </c>
       <c r="E147" s="3"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>158</v>
       </c>
@@ -3541,7 +3542,7 @@
       </c>
       <c r="E148" s="3"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>158</v>
       </c>
@@ -3556,7 +3557,7 @@
       </c>
       <c r="E149" s="3"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>158</v>
       </c>
@@ -3571,7 +3572,7 @@
       </c>
       <c r="E150" s="3"/>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>158</v>
       </c>
@@ -3586,7 +3587,7 @@
       </c>
       <c r="E151" s="3"/>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>158</v>
       </c>
@@ -3601,7 +3602,7 @@
       </c>
       <c r="E152" s="3"/>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>158</v>
       </c>
@@ -3616,7 +3617,7 @@
       </c>
       <c r="E153" s="3"/>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>158</v>
       </c>
@@ -3631,7 +3632,7 @@
       </c>
       <c r="E154" s="3"/>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>158</v>
       </c>
@@ -3646,7 +3647,7 @@
       </c>
       <c r="E155" s="3"/>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>158</v>
       </c>
@@ -3661,7 +3662,7 @@
       </c>
       <c r="E156" s="3"/>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>158</v>
       </c>
@@ -3676,7 +3677,7 @@
       </c>
       <c r="E157" s="3"/>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>158</v>
       </c>
@@ -3691,7 +3692,7 @@
       </c>
       <c r="E158" s="3"/>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>158</v>
       </c>
@@ -3706,7 +3707,7 @@
       </c>
       <c r="E159" s="3"/>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>158</v>
       </c>
@@ -3721,7 +3722,7 @@
       </c>
       <c r="E160" s="3"/>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>158</v>
       </c>
@@ -3736,7 +3737,7 @@
       </c>
       <c r="E161" s="3"/>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>158</v>
       </c>
@@ -3751,7 +3752,7 @@
       </c>
       <c r="E162" s="3"/>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>158</v>
       </c>
@@ -3766,7 +3767,7 @@
       </c>
       <c r="E163" s="3"/>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>158</v>
       </c>
@@ -3781,7 +3782,7 @@
       </c>
       <c r="E164" s="3"/>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>158</v>
       </c>
@@ -3796,7 +3797,7 @@
       </c>
       <c r="E165" s="3"/>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>158</v>
       </c>
@@ -3811,7 +3812,7 @@
       </c>
       <c r="E166" s="3"/>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>158</v>
       </c>
@@ -3826,7 +3827,7 @@
       </c>
       <c r="E167" s="3"/>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>158</v>
       </c>
@@ -3841,7 +3842,7 @@
       </c>
       <c r="E168" s="3"/>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>158</v>
       </c>
@@ -3856,7 +3857,7 @@
       </c>
       <c r="E169" s="3"/>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>158</v>
       </c>
@@ -3871,7 +3872,7 @@
       </c>
       <c r="E170" s="3"/>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>158</v>
       </c>
@@ -3886,7 +3887,7 @@
       </c>
       <c r="E171" s="3"/>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>158</v>
       </c>
@@ -3901,7 +3902,7 @@
       </c>
       <c r="E172" s="3"/>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>158</v>
       </c>
@@ -3916,7 +3917,7 @@
       </c>
       <c r="E173" s="3"/>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>158</v>
       </c>
@@ -3931,7 +3932,7 @@
       </c>
       <c r="E174" s="3"/>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>158</v>
       </c>
@@ -3946,7 +3947,7 @@
       </c>
       <c r="E175" s="3"/>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>158</v>
       </c>
@@ -3961,7 +3962,7 @@
       </c>
       <c r="E176" s="3"/>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>158</v>
       </c>
@@ -3976,7 +3977,7 @@
       </c>
       <c r="E177" s="3"/>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>158</v>
       </c>
@@ -3991,7 +3992,7 @@
       </c>
       <c r="E178" s="3"/>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>158</v>
       </c>
@@ -4006,7 +4007,7 @@
       </c>
       <c r="E179" s="3"/>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>158</v>
       </c>
@@ -4021,7 +4022,7 @@
       </c>
       <c r="E180" s="3"/>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>158</v>
       </c>
@@ -4036,7 +4037,7 @@
       </c>
       <c r="E181" s="3"/>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>158</v>
       </c>
@@ -4051,7 +4052,7 @@
       </c>
       <c r="E182" s="3"/>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>158</v>
       </c>
@@ -4066,7 +4067,7 @@
       </c>
       <c r="E183" s="3"/>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>158</v>
       </c>
@@ -4081,7 +4082,7 @@
       </c>
       <c r="E184" s="3"/>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>158</v>
       </c>
@@ -4096,7 +4097,7 @@
       </c>
       <c r="E185" s="3"/>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>158</v>
       </c>
@@ -4111,7 +4112,7 @@
       </c>
       <c r="E186" s="3"/>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>158</v>
       </c>
@@ -4126,7 +4127,7 @@
       </c>
       <c r="E187" s="3"/>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>158</v>
       </c>
@@ -4141,7 +4142,7 @@
       </c>
       <c r="E188" s="3"/>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>158</v>
       </c>
@@ -4156,7 +4157,7 @@
       </c>
       <c r="E189" s="3"/>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>158</v>
       </c>
@@ -4171,7 +4172,7 @@
       </c>
       <c r="E190" s="3"/>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>158</v>
       </c>
@@ -4186,7 +4187,7 @@
       </c>
       <c r="E191" s="3"/>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>158</v>
       </c>
@@ -4201,7 +4202,7 @@
       </c>
       <c r="E192" s="3"/>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>158</v>
       </c>
@@ -4216,7 +4217,7 @@
       </c>
       <c r="E193" s="3"/>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>158</v>
       </c>
@@ -4231,7 +4232,7 @@
       </c>
       <c r="E194" s="3"/>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>158</v>
       </c>
@@ -4246,7 +4247,7 @@
       </c>
       <c r="E195" s="3"/>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>158</v>
       </c>
@@ -4261,7 +4262,7 @@
       </c>
       <c r="E196" s="3"/>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>158</v>
       </c>
@@ -4276,7 +4277,7 @@
       </c>
       <c r="E197" s="3"/>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>158</v>
       </c>
@@ -4291,7 +4292,7 @@
       </c>
       <c r="E198" s="3"/>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>158</v>
       </c>
@@ -4306,7 +4307,7 @@
       </c>
       <c r="E199" s="3"/>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>158</v>
       </c>
@@ -4321,7 +4322,7 @@
       </c>
       <c r="E200" s="3"/>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>158</v>
       </c>
@@ -4336,7 +4337,7 @@
       </c>
       <c r="E201" s="3"/>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>158</v>
       </c>
@@ -4351,7 +4352,7 @@
       </c>
       <c r="E202" s="3"/>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>158</v>
       </c>
@@ -4366,7 +4367,7 @@
       </c>
       <c r="E203" s="3"/>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>158</v>
       </c>
@@ -4381,7 +4382,7 @@
       </c>
       <c r="E204" s="3"/>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>158</v>
       </c>
@@ -4396,7 +4397,7 @@
       </c>
       <c r="E205" s="3"/>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>158</v>
       </c>
@@ -4411,7 +4412,7 @@
       </c>
       <c r="E206" s="3"/>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>158</v>
       </c>
@@ -4426,7 +4427,7 @@
       </c>
       <c r="E207" s="3"/>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>158</v>
       </c>
@@ -4441,7 +4442,7 @@
       </c>
       <c r="E208" s="3"/>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>158</v>
       </c>
@@ -4456,7 +4457,7 @@
       </c>
       <c r="E209" s="3"/>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>158</v>
       </c>
@@ -4471,7 +4472,7 @@
       </c>
       <c r="E210" s="3"/>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>158</v>
       </c>
@@ -4486,7 +4487,7 @@
       </c>
       <c r="E211" s="3"/>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>158</v>
       </c>
@@ -4501,7 +4502,7 @@
       </c>
       <c r="E212" s="3"/>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>158</v>
       </c>
@@ -4516,7 +4517,7 @@
       </c>
       <c r="E213" s="3"/>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>158</v>
       </c>
@@ -4531,7 +4532,7 @@
       </c>
       <c r="E214" s="3"/>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>158</v>
       </c>
@@ -4546,7 +4547,7 @@
       </c>
       <c r="E215" s="3"/>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>158</v>
       </c>
@@ -4561,7 +4562,7 @@
       </c>
       <c r="E216" s="3"/>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>158</v>
       </c>
@@ -4576,7 +4577,7 @@
       </c>
       <c r="E217" s="3"/>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>158</v>
       </c>
@@ -4591,7 +4592,7 @@
       </c>
       <c r="E218" s="3"/>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>158</v>
       </c>
@@ -4606,7 +4607,7 @@
       </c>
       <c r="E219" s="3"/>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>158</v>
       </c>
@@ -4622,15 +4623,15 @@
       <c r="E220" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E220" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E220"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -4670,7 +4671,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" ht="14.4" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -4681,7 +4682,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" ht="14.4" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -4957,7 +4958,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C29" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Started with Two pointers
</commit_message>
<xml_diff>
--- a/Java_Developer_Roadmap.xlsx
+++ b/Java_Developer_Roadmap.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{094BE57E-1E2E-497B-9B9A-398F3C083BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Roadmap" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Topics &amp; Subtopics" state="visible" r:id="rId5"/>
+    <sheet name="Roadmap" sheetId="1" r:id="rId1"/>
+    <sheet name="Topics &amp; Subtopics" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">'Topics &amp; Subtopics'!$A$1:$C$29</definedName>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="288">
   <si>
     <t>Level</t>
   </si>
@@ -887,19 +888,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1245,9 +1246,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E220"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -1817,7 +1818,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>26</v>
       </c>
@@ -1830,7 +1831,9 @@
       <c r="D34" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E34" s="3"/>
+      <c r="E34" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
@@ -1937,7 +1940,7 @@
       </c>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>26</v>
       </c>
@@ -1952,7 +1955,7 @@
       </c>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>26</v>
       </c>
@@ -1967,7 +1970,7 @@
       </c>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>26</v>
       </c>
@@ -1982,7 +1985,7 @@
       </c>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>26</v>
       </c>
@@ -1997,7 +2000,7 @@
       </c>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2012,7 +2015,7 @@
       </c>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>26</v>
       </c>
@@ -2027,7 +2030,7 @@
       </c>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>26</v>
       </c>
@@ -2042,7 +2045,7 @@
       </c>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>61</v>
       </c>
@@ -2057,7 +2060,7 @@
       </c>
       <c r="E49" s="3"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>61</v>
       </c>
@@ -2072,7 +2075,7 @@
       </c>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>61</v>
       </c>
@@ -2087,7 +2090,7 @@
       </c>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>61</v>
       </c>
@@ -2102,7 +2105,7 @@
       </c>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>61</v>
       </c>
@@ -2117,7 +2120,7 @@
       </c>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>61</v>
       </c>
@@ -2132,7 +2135,7 @@
       </c>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>61</v>
       </c>
@@ -2147,7 +2150,7 @@
       </c>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>61</v>
       </c>
@@ -2162,7 +2165,7 @@
       </c>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>61</v>
       </c>
@@ -2177,7 +2180,7 @@
       </c>
       <c r="E57" s="3"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>61</v>
       </c>
@@ -2192,7 +2195,7 @@
       </c>
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>61</v>
       </c>
@@ -2207,7 +2210,7 @@
       </c>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>61</v>
       </c>
@@ -2222,7 +2225,7 @@
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>61</v>
       </c>
@@ -2237,7 +2240,7 @@
       </c>
       <c r="E61" s="3"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -2252,7 +2255,7 @@
       </c>
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -2267,7 +2270,7 @@
       </c>
       <c r="E63" s="3"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>61</v>
       </c>
@@ -2282,7 +2285,7 @@
       </c>
       <c r="E64" s="3"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>61</v>
       </c>
@@ -2297,7 +2300,7 @@
       </c>
       <c r="E65" s="3"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>61</v>
       </c>
@@ -2312,7 +2315,7 @@
       </c>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>61</v>
       </c>
@@ -2327,7 +2330,7 @@
       </c>
       <c r="E67" s="3"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>61</v>
       </c>
@@ -2342,7 +2345,7 @@
       </c>
       <c r="E68" s="3"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>61</v>
       </c>
@@ -2357,7 +2360,7 @@
       </c>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>61</v>
       </c>
@@ -2372,7 +2375,7 @@
       </c>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>61</v>
       </c>
@@ -2387,7 +2390,7 @@
       </c>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>61</v>
       </c>
@@ -2402,7 +2405,7 @@
       </c>
       <c r="E72" s="3"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>61</v>
       </c>
@@ -2417,7 +2420,7 @@
       </c>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>61</v>
       </c>
@@ -2432,7 +2435,7 @@
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>61</v>
       </c>
@@ -2447,7 +2450,7 @@
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>61</v>
       </c>
@@ -2462,7 +2465,7 @@
       </c>
       <c r="E76" s="3"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>61</v>
       </c>
@@ -2477,7 +2480,7 @@
       </c>
       <c r="E77" s="3"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>61</v>
       </c>
@@ -2492,7 +2495,7 @@
       </c>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>61</v>
       </c>
@@ -2507,7 +2510,7 @@
       </c>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>61</v>
       </c>
@@ -2522,7 +2525,7 @@
       </c>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>61</v>
       </c>
@@ -2537,7 +2540,7 @@
       </c>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>61</v>
       </c>
@@ -2552,7 +2555,7 @@
       </c>
       <c r="E82" s="3"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>61</v>
       </c>
@@ -2567,7 +2570,7 @@
       </c>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>61</v>
       </c>
@@ -2582,7 +2585,7 @@
       </c>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>61</v>
       </c>
@@ -2597,7 +2600,7 @@
       </c>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>61</v>
       </c>
@@ -2612,7 +2615,7 @@
       </c>
       <c r="E86" s="3"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>61</v>
       </c>
@@ -2627,7 +2630,7 @@
       </c>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>61</v>
       </c>
@@ -2642,7 +2645,7 @@
       </c>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>61</v>
       </c>
@@ -2657,7 +2660,7 @@
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>61</v>
       </c>
@@ -2672,7 +2675,7 @@
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>61</v>
       </c>
@@ -2687,7 +2690,7 @@
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>61</v>
       </c>
@@ -2702,7 +2705,7 @@
       </c>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>61</v>
       </c>
@@ -2717,7 +2720,7 @@
       </c>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>61</v>
       </c>
@@ -2732,7 +2735,7 @@
       </c>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>61</v>
       </c>
@@ -2747,7 +2750,7 @@
       </c>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>61</v>
       </c>
@@ -2762,7 +2765,7 @@
       </c>
       <c r="E96" s="3"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>61</v>
       </c>
@@ -2777,7 +2780,7 @@
       </c>
       <c r="E97" s="3"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>61</v>
       </c>
@@ -2792,7 +2795,7 @@
       </c>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>61</v>
       </c>
@@ -2807,7 +2810,7 @@
       </c>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>61</v>
       </c>
@@ -2822,7 +2825,7 @@
       </c>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>120</v>
       </c>
@@ -2837,7 +2840,7 @@
       </c>
       <c r="E101" s="3"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>120</v>
       </c>
@@ -2852,7 +2855,7 @@
       </c>
       <c r="E102" s="3"/>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>120</v>
       </c>
@@ -2867,7 +2870,7 @@
       </c>
       <c r="E103" s="3"/>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>120</v>
       </c>
@@ -2882,7 +2885,7 @@
       </c>
       <c r="E104" s="3"/>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>120</v>
       </c>
@@ -2897,7 +2900,7 @@
       </c>
       <c r="E105" s="3"/>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>120</v>
       </c>
@@ -2912,7 +2915,7 @@
       </c>
       <c r="E106" s="3"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>120</v>
       </c>
@@ -2927,7 +2930,7 @@
       </c>
       <c r="E107" s="3"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>120</v>
       </c>
@@ -2942,7 +2945,7 @@
       </c>
       <c r="E108" s="3"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>120</v>
       </c>
@@ -2957,7 +2960,7 @@
       </c>
       <c r="E109" s="3"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>120</v>
       </c>
@@ -2972,7 +2975,7 @@
       </c>
       <c r="E110" s="3"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>120</v>
       </c>
@@ -2987,7 +2990,7 @@
       </c>
       <c r="E111" s="3"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>120</v>
       </c>
@@ -3002,7 +3005,7 @@
       </c>
       <c r="E112" s="3"/>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>120</v>
       </c>
@@ -3017,7 +3020,7 @@
       </c>
       <c r="E113" s="3"/>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>120</v>
       </c>
@@ -3032,7 +3035,7 @@
       </c>
       <c r="E114" s="3"/>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>120</v>
       </c>
@@ -3047,7 +3050,7 @@
       </c>
       <c r="E115" s="3"/>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>120</v>
       </c>
@@ -3062,7 +3065,7 @@
       </c>
       <c r="E116" s="3"/>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>120</v>
       </c>
@@ -3077,7 +3080,7 @@
       </c>
       <c r="E117" s="3"/>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>120</v>
       </c>
@@ -3092,7 +3095,7 @@
       </c>
       <c r="E118" s="3"/>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>120</v>
       </c>
@@ -3107,7 +3110,7 @@
       </c>
       <c r="E119" s="3"/>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>120</v>
       </c>
@@ -3122,7 +3125,7 @@
       </c>
       <c r="E120" s="3"/>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>120</v>
       </c>
@@ -3137,7 +3140,7 @@
       </c>
       <c r="E121" s="3"/>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>120</v>
       </c>
@@ -3152,7 +3155,7 @@
       </c>
       <c r="E122" s="3"/>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>120</v>
       </c>
@@ -3167,7 +3170,7 @@
       </c>
       <c r="E123" s="3"/>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>120</v>
       </c>
@@ -3182,7 +3185,7 @@
       </c>
       <c r="E124" s="3"/>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>120</v>
       </c>
@@ -3197,7 +3200,7 @@
       </c>
       <c r="E125" s="3"/>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>120</v>
       </c>
@@ -3212,7 +3215,7 @@
       </c>
       <c r="E126" s="3"/>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>120</v>
       </c>
@@ -3227,7 +3230,7 @@
       </c>
       <c r="E127" s="3"/>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>120</v>
       </c>
@@ -3242,7 +3245,7 @@
       </c>
       <c r="E128" s="3"/>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>120</v>
       </c>
@@ -3257,7 +3260,7 @@
       </c>
       <c r="E129" s="3"/>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>120</v>
       </c>
@@ -3272,7 +3275,7 @@
       </c>
       <c r="E130" s="3"/>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>120</v>
       </c>
@@ -3287,7 +3290,7 @@
       </c>
       <c r="E131" s="3"/>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>120</v>
       </c>
@@ -3302,7 +3305,7 @@
       </c>
       <c r="E132" s="3"/>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>158</v>
       </c>
@@ -3317,7 +3320,7 @@
       </c>
       <c r="E133" s="3"/>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>158</v>
       </c>
@@ -3332,7 +3335,7 @@
       </c>
       <c r="E134" s="3"/>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>158</v>
       </c>
@@ -3347,7 +3350,7 @@
       </c>
       <c r="E135" s="3"/>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>158</v>
       </c>
@@ -3362,7 +3365,7 @@
       </c>
       <c r="E136" s="3"/>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>158</v>
       </c>
@@ -3377,7 +3380,7 @@
       </c>
       <c r="E137" s="3"/>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>158</v>
       </c>
@@ -3392,7 +3395,7 @@
       </c>
       <c r="E138" s="3"/>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>158</v>
       </c>
@@ -3407,7 +3410,7 @@
       </c>
       <c r="E139" s="3"/>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>158</v>
       </c>
@@ -3422,7 +3425,7 @@
       </c>
       <c r="E140" s="3"/>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>158</v>
       </c>
@@ -3437,7 +3440,7 @@
       </c>
       <c r="E141" s="3"/>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>158</v>
       </c>
@@ -3452,7 +3455,7 @@
       </c>
       <c r="E142" s="3"/>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>158</v>
       </c>
@@ -3467,7 +3470,7 @@
       </c>
       <c r="E143" s="3"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>158</v>
       </c>
@@ -3482,7 +3485,7 @@
       </c>
       <c r="E144" s="3"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>158</v>
       </c>
@@ -3497,7 +3500,7 @@
       </c>
       <c r="E145" s="3"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>158</v>
       </c>
@@ -3512,7 +3515,7 @@
       </c>
       <c r="E146" s="3"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>158</v>
       </c>
@@ -3527,7 +3530,7 @@
       </c>
       <c r="E147" s="3"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>158</v>
       </c>
@@ -3542,7 +3545,7 @@
       </c>
       <c r="E148" s="3"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>158</v>
       </c>
@@ -3557,7 +3560,7 @@
       </c>
       <c r="E149" s="3"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>158</v>
       </c>
@@ -3572,7 +3575,7 @@
       </c>
       <c r="E150" s="3"/>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>158</v>
       </c>
@@ -3587,7 +3590,7 @@
       </c>
       <c r="E151" s="3"/>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>158</v>
       </c>
@@ -3602,7 +3605,7 @@
       </c>
       <c r="E152" s="3"/>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>158</v>
       </c>
@@ -3617,7 +3620,7 @@
       </c>
       <c r="E153" s="3"/>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>158</v>
       </c>
@@ -3632,7 +3635,7 @@
       </c>
       <c r="E154" s="3"/>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>158</v>
       </c>
@@ -3647,7 +3650,7 @@
       </c>
       <c r="E155" s="3"/>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>158</v>
       </c>
@@ -3662,7 +3665,7 @@
       </c>
       <c r="E156" s="3"/>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>158</v>
       </c>
@@ -3677,7 +3680,7 @@
       </c>
       <c r="E157" s="3"/>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
         <v>158</v>
       </c>
@@ -3692,7 +3695,7 @@
       </c>
       <c r="E158" s="3"/>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
         <v>158</v>
       </c>
@@ -3707,7 +3710,7 @@
       </c>
       <c r="E159" s="3"/>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
         <v>158</v>
       </c>
@@ -3722,7 +3725,7 @@
       </c>
       <c r="E160" s="3"/>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
         <v>158</v>
       </c>
@@ -3737,7 +3740,7 @@
       </c>
       <c r="E161" s="3"/>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>158</v>
       </c>
@@ -3752,7 +3755,7 @@
       </c>
       <c r="E162" s="3"/>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
         <v>158</v>
       </c>
@@ -3767,7 +3770,7 @@
       </c>
       <c r="E163" s="3"/>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
         <v>158</v>
       </c>
@@ -3782,7 +3785,7 @@
       </c>
       <c r="E164" s="3"/>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
         <v>158</v>
       </c>
@@ -3797,7 +3800,7 @@
       </c>
       <c r="E165" s="3"/>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
         <v>158</v>
       </c>
@@ -3812,7 +3815,7 @@
       </c>
       <c r="E166" s="3"/>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>158</v>
       </c>
@@ -3827,7 +3830,7 @@
       </c>
       <c r="E167" s="3"/>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
         <v>158</v>
       </c>
@@ -3842,7 +3845,7 @@
       </c>
       <c r="E168" s="3"/>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
         <v>158</v>
       </c>
@@ -3857,7 +3860,7 @@
       </c>
       <c r="E169" s="3"/>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
         <v>158</v>
       </c>
@@ -3872,7 +3875,7 @@
       </c>
       <c r="E170" s="3"/>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
         <v>158</v>
       </c>
@@ -3887,7 +3890,7 @@
       </c>
       <c r="E171" s="3"/>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>158</v>
       </c>
@@ -3902,7 +3905,7 @@
       </c>
       <c r="E172" s="3"/>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>158</v>
       </c>
@@ -3917,7 +3920,7 @@
       </c>
       <c r="E173" s="3"/>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>158</v>
       </c>
@@ -3932,7 +3935,7 @@
       </c>
       <c r="E174" s="3"/>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>158</v>
       </c>
@@ -3947,7 +3950,7 @@
       </c>
       <c r="E175" s="3"/>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>158</v>
       </c>
@@ -3962,7 +3965,7 @@
       </c>
       <c r="E176" s="3"/>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>158</v>
       </c>
@@ -3977,7 +3980,7 @@
       </c>
       <c r="E177" s="3"/>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>158</v>
       </c>
@@ -3992,7 +3995,7 @@
       </c>
       <c r="E178" s="3"/>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>158</v>
       </c>
@@ -4007,7 +4010,7 @@
       </c>
       <c r="E179" s="3"/>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>158</v>
       </c>
@@ -4022,7 +4025,7 @@
       </c>
       <c r="E180" s="3"/>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>158</v>
       </c>
@@ -4037,7 +4040,7 @@
       </c>
       <c r="E181" s="3"/>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>158</v>
       </c>
@@ -4052,7 +4055,7 @@
       </c>
       <c r="E182" s="3"/>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
         <v>158</v>
       </c>
@@ -4067,7 +4070,7 @@
       </c>
       <c r="E183" s="3"/>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
         <v>158</v>
       </c>
@@ -4082,7 +4085,7 @@
       </c>
       <c r="E184" s="3"/>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
         <v>158</v>
       </c>
@@ -4097,7 +4100,7 @@
       </c>
       <c r="E185" s="3"/>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
         <v>158</v>
       </c>
@@ -4112,7 +4115,7 @@
       </c>
       <c r="E186" s="3"/>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>158</v>
       </c>
@@ -4127,7 +4130,7 @@
       </c>
       <c r="E187" s="3"/>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
         <v>158</v>
       </c>
@@ -4142,7 +4145,7 @@
       </c>
       <c r="E188" s="3"/>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
         <v>158</v>
       </c>
@@ -4157,7 +4160,7 @@
       </c>
       <c r="E189" s="3"/>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
         <v>158</v>
       </c>
@@ -4172,7 +4175,7 @@
       </c>
       <c r="E190" s="3"/>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
         <v>158</v>
       </c>
@@ -4187,7 +4190,7 @@
       </c>
       <c r="E191" s="3"/>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>158</v>
       </c>
@@ -4202,7 +4205,7 @@
       </c>
       <c r="E192" s="3"/>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
         <v>158</v>
       </c>
@@ -4217,7 +4220,7 @@
       </c>
       <c r="E193" s="3"/>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
         <v>158</v>
       </c>
@@ -4232,7 +4235,7 @@
       </c>
       <c r="E194" s="3"/>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
         <v>158</v>
       </c>
@@ -4247,7 +4250,7 @@
       </c>
       <c r="E195" s="3"/>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
         <v>158</v>
       </c>
@@ -4262,7 +4265,7 @@
       </c>
       <c r="E196" s="3"/>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>158</v>
       </c>
@@ -4277,7 +4280,7 @@
       </c>
       <c r="E197" s="3"/>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>158</v>
       </c>
@@ -4292,7 +4295,7 @@
       </c>
       <c r="E198" s="3"/>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
         <v>158</v>
       </c>
@@ -4307,7 +4310,7 @@
       </c>
       <c r="E199" s="3"/>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
         <v>158</v>
       </c>
@@ -4322,7 +4325,7 @@
       </c>
       <c r="E200" s="3"/>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
         <v>158</v>
       </c>
@@ -4337,7 +4340,7 @@
       </c>
       <c r="E201" s="3"/>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>158</v>
       </c>
@@ -4352,7 +4355,7 @@
       </c>
       <c r="E202" s="3"/>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
         <v>158</v>
       </c>
@@ -4367,7 +4370,7 @@
       </c>
       <c r="E203" s="3"/>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
         <v>158</v>
       </c>
@@ -4382,7 +4385,7 @@
       </c>
       <c r="E204" s="3"/>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
         <v>158</v>
       </c>
@@ -4397,7 +4400,7 @@
       </c>
       <c r="E205" s="3"/>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
         <v>158</v>
       </c>
@@ -4412,7 +4415,7 @@
       </c>
       <c r="E206" s="3"/>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>158</v>
       </c>
@@ -4427,7 +4430,7 @@
       </c>
       <c r="E207" s="3"/>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
         <v>158</v>
       </c>
@@ -4442,7 +4445,7 @@
       </c>
       <c r="E208" s="3"/>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
         <v>158</v>
       </c>
@@ -4457,7 +4460,7 @@
       </c>
       <c r="E209" s="3"/>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>158</v>
       </c>
@@ -4472,7 +4475,7 @@
       </c>
       <c r="E210" s="3"/>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>158</v>
       </c>
@@ -4487,7 +4490,7 @@
       </c>
       <c r="E211" s="3"/>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>158</v>
       </c>
@@ -4502,7 +4505,7 @@
       </c>
       <c r="E212" s="3"/>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>158</v>
       </c>
@@ -4517,7 +4520,7 @@
       </c>
       <c r="E213" s="3"/>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>158</v>
       </c>
@@ -4532,7 +4535,7 @@
       </c>
       <c r="E214" s="3"/>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>158</v>
       </c>
@@ -4547,7 +4550,7 @@
       </c>
       <c r="E215" s="3"/>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
         <v>158</v>
       </c>
@@ -4562,7 +4565,7 @@
       </c>
       <c r="E216" s="3"/>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>158</v>
       </c>
@@ -4577,7 +4580,7 @@
       </c>
       <c r="E217" s="3"/>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
         <v>158</v>
       </c>
@@ -4592,7 +4595,7 @@
       </c>
       <c r="E218" s="3"/>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
         <v>158</v>
       </c>
@@ -4607,7 +4610,7 @@
       </c>
       <c r="E219" s="3"/>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
         <v>158</v>
       </c>
@@ -4623,15 +4626,15 @@
       <c r="E220" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E220"/>
+  <autoFilter ref="A1:E220" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -4671,7 +4674,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" ht="14.4" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -4682,7 +4685,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="5" ht="14.4" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -4958,7 +4961,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C29"/>
+  <autoFilter ref="A1:C29" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>